<commit_message>
Actualizacion automatica de datos desde el Boton Magico
</commit_message>
<xml_diff>
--- a/data/EVALUACIONES/AEROBICO/AEROBICO_5MIN.xlsx
+++ b/data/EVALUACIONES/AEROBICO/AEROBICO_5MIN.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30416"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\ADARVE JUV D.H\App_Rendimiento_Futbol\data\EVALUACIONES\AEROBICO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{70C7CA30-4A11-43CA-A210-8E38ACFDF285}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5A30F84B-0D3B-43C3-BC3B-59CE6A14E4BB}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{70C7CA30-4A11-43CA-A210-8E38ACFDF285}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{78C8FB91-492F-4B55-A8AC-7EDC7FBDD265}"/>
   <bookViews>
-    <workbookView xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="9960" xr2:uid="{BBC13A56-B43E-4445-9420-3EF783FE99BE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{BBC13A56-B43E-4445-9420-3EF783FE99BE}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="32">
   <si>
     <t>Fecha</t>
   </si>
@@ -58,9 +58,6 @@
   </si>
   <si>
     <t>Ikki_Muller_Salak</t>
-  </si>
-  <si>
-    <t>Alejandro_Garcia_Gumiel</t>
   </si>
   <si>
     <t>Rodri_Sanchez_Ramos</t>
@@ -220,8 +217,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{47DCDBC4-934F-4BB8-8403-1163E6A946CF}" name="Tabla1" displayName="Tabla1" ref="A1:E76" totalsRowShown="0" headerRowDxfId="2">
-  <autoFilter ref="A1:E76" xr:uid="{F24D9BFF-4F02-4AC6-9C99-CC9D7330899E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{47DCDBC4-934F-4BB8-8403-1163E6A946CF}" name="Tabla1" displayName="Tabla1" ref="A1:E73" totalsRowShown="0" headerRowDxfId="2">
+  <autoFilter ref="A1:E73" xr:uid="{F24D9BFF-4F02-4AC6-9C99-CC9D7330899E}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{B90CC2EA-DED7-4B50-9C01-6648707B7686}" name="Fecha" dataDxfId="1"/>
     <tableColumn id="2" xr3:uid="{49BFBD1B-88C4-49EF-ACC0-907CF6D29923}" name="Nombre"/>
@@ -530,7 +527,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FF0B100-72AE-4E6A-8897-D79B621AF892}">
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:E73"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="28.5546875" bestFit="1" customWidth="1"/>
@@ -559,7 +556,7 @@
         <v>46204</v>
       </c>
       <c r="B2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C2">
         <v>1.34</v>
@@ -684,15 +681,12 @@
       <c r="B9" t="s">
         <v>11</v>
       </c>
-      <c r="C9">
-        <v>1.2</v>
-      </c>
       <c r="D9">
         <v>5</v>
       </c>
       <c r="E9" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>14.399999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
@@ -702,12 +696,15 @@
       <c r="B10" t="s">
         <v>12</v>
       </c>
+      <c r="C10">
+        <v>1.41</v>
+      </c>
       <c r="D10">
         <v>5</v>
       </c>
       <c r="E10" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>0</v>
+        <v>16.919999999999998</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
@@ -718,14 +715,14 @@
         <v>13</v>
       </c>
       <c r="C11">
-        <v>1.41</v>
+        <v>1.36</v>
       </c>
       <c r="D11">
         <v>5</v>
       </c>
       <c r="E11" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>16.919999999999998</v>
+        <v>16.32</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
@@ -735,15 +732,12 @@
       <c r="B12" t="s">
         <v>14</v>
       </c>
-      <c r="C12">
-        <v>1.36</v>
-      </c>
       <c r="D12">
         <v>5</v>
       </c>
       <c r="E12" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>16.32</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
@@ -753,12 +747,15 @@
       <c r="B13" t="s">
         <v>15</v>
       </c>
+      <c r="C13">
+        <v>1.33</v>
+      </c>
       <c r="D13">
         <v>5</v>
       </c>
       <c r="E13" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>0</v>
+        <v>15.96</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
@@ -769,14 +766,14 @@
         <v>16</v>
       </c>
       <c r="C14">
-        <v>1.33</v>
+        <v>1.34</v>
       </c>
       <c r="D14">
         <v>5</v>
       </c>
       <c r="E14" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>15.96</v>
+        <v>16.080000000000002</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
@@ -787,14 +784,14 @@
         <v>17</v>
       </c>
       <c r="C15">
-        <v>1.34</v>
+        <v>1.37</v>
       </c>
       <c r="D15">
         <v>5</v>
       </c>
       <c r="E15" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>16.080000000000002</v>
+        <v>16.440000000000001</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
@@ -805,14 +802,14 @@
         <v>18</v>
       </c>
       <c r="C16">
-        <v>1.37</v>
+        <v>1.33</v>
       </c>
       <c r="D16">
         <v>5</v>
       </c>
       <c r="E16" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>16.440000000000001</v>
+        <v>15.96</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
@@ -823,14 +820,14 @@
         <v>19</v>
       </c>
       <c r="C17">
-        <v>1.33</v>
+        <v>1.35</v>
       </c>
       <c r="D17">
         <v>5</v>
       </c>
       <c r="E17" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>15.96</v>
+        <v>16.200000000000003</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
@@ -840,15 +837,12 @@
       <c r="B18" t="s">
         <v>20</v>
       </c>
-      <c r="C18">
-        <v>1.35</v>
-      </c>
       <c r="D18">
         <v>5</v>
       </c>
       <c r="E18" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>16.200000000000003</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
@@ -858,12 +852,15 @@
       <c r="B19" t="s">
         <v>21</v>
       </c>
+      <c r="C19">
+        <v>1.1499999999999999</v>
+      </c>
       <c r="D19">
         <v>5</v>
       </c>
       <c r="E19" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>0</v>
+        <v>13.799999999999999</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
@@ -874,14 +871,14 @@
         <v>22</v>
       </c>
       <c r="C20">
-        <v>1.1499999999999999</v>
+        <v>1.31</v>
       </c>
       <c r="D20">
         <v>5</v>
       </c>
       <c r="E20" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>13.799999999999999</v>
+        <v>15.72</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
@@ -892,14 +889,14 @@
         <v>23</v>
       </c>
       <c r="C21">
-        <v>1.31</v>
+        <v>1.35</v>
       </c>
       <c r="D21">
         <v>5</v>
       </c>
       <c r="E21" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>15.72</v>
+        <v>16.200000000000003</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
@@ -910,50 +907,50 @@
         <v>24</v>
       </c>
       <c r="C22">
-        <v>1.35</v>
+        <v>1.5</v>
       </c>
       <c r="D22">
         <v>5</v>
       </c>
       <c r="E22" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>16.200000000000003</v>
+        <v>18</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <v>46204</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="4" t="s">
         <v>25</v>
       </c>
       <c r="C23">
-        <v>1.5</v>
+        <v>0.86</v>
       </c>
       <c r="D23">
         <v>5</v>
       </c>
       <c r="E23" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>18</v>
+        <v>10.319999999999999</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>46204</v>
       </c>
-      <c r="B24" s="4" t="s">
-        <v>26</v>
+      <c r="B24" t="s">
+        <v>29</v>
       </c>
       <c r="C24">
-        <v>0.86</v>
+        <v>1.33</v>
       </c>
       <c r="D24">
         <v>5</v>
       </c>
       <c r="E24" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>10.319999999999999</v>
+        <v>15.96</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
@@ -961,17 +958,14 @@
         <v>46204</v>
       </c>
       <c r="B25" t="s">
-        <v>30</v>
-      </c>
-      <c r="C25">
-        <v>1.33</v>
+        <v>26</v>
       </c>
       <c r="D25">
         <v>5</v>
       </c>
       <c r="E25" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>15.96</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
@@ -979,14 +973,17 @@
         <v>46204</v>
       </c>
       <c r="B26" t="s">
-        <v>27</v>
+        <v>30</v>
+      </c>
+      <c r="C26">
+        <v>1.19</v>
       </c>
       <c r="D26">
         <v>5</v>
       </c>
       <c r="E26" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>0</v>
+        <v>14.28</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
@@ -994,32 +991,32 @@
         <v>46204</v>
       </c>
       <c r="B27" t="s">
-        <v>31</v>
-      </c>
-      <c r="C27">
-        <v>1.19</v>
+        <v>27</v>
       </c>
       <c r="D27">
         <v>5</v>
       </c>
       <c r="E27" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>14.28</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
-        <v>46204</v>
+        <v>46247</v>
       </c>
       <c r="B28" t="s">
-        <v>28</v>
+        <v>5</v>
+      </c>
+      <c r="C28">
+        <v>1.38</v>
       </c>
       <c r="D28">
         <v>5</v>
       </c>
       <c r="E28" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>0</v>
+        <v>16.559999999999999</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
@@ -1027,17 +1024,17 @@
         <v>46247</v>
       </c>
       <c r="B29" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C29">
-        <v>1.38</v>
+        <v>1.44</v>
       </c>
       <c r="D29">
         <v>5</v>
       </c>
       <c r="E29" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>16.559999999999999</v>
+        <v>17.279999999999998</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
@@ -1045,17 +1042,17 @@
         <v>46247</v>
       </c>
       <c r="B30" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C30">
-        <v>1.44</v>
+        <v>1.34</v>
       </c>
       <c r="D30">
         <v>5</v>
       </c>
       <c r="E30" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>17.279999999999998</v>
+        <v>16.080000000000002</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
@@ -1063,17 +1060,17 @@
         <v>46247</v>
       </c>
       <c r="B31" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C31">
-        <v>1.34</v>
+        <v>1.51</v>
       </c>
       <c r="D31">
         <v>5</v>
       </c>
       <c r="E31" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>16.080000000000002</v>
+        <v>18.12</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
@@ -1081,17 +1078,17 @@
         <v>46247</v>
       </c>
       <c r="B32" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C32">
-        <v>1.51</v>
+        <v>1.35</v>
       </c>
       <c r="D32">
         <v>5</v>
       </c>
       <c r="E32" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>18.12</v>
+        <v>16.200000000000003</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
@@ -1099,17 +1096,17 @@
         <v>46247</v>
       </c>
       <c r="B33" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C33">
-        <v>1.35</v>
+        <v>1.54</v>
       </c>
       <c r="D33">
         <v>5</v>
       </c>
       <c r="E33" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>16.200000000000003</v>
+        <v>18.48</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
@@ -1117,17 +1114,14 @@
         <v>46247</v>
       </c>
       <c r="B34" t="s">
-        <v>10</v>
-      </c>
-      <c r="C34">
-        <v>1.54</v>
+        <v>11</v>
       </c>
       <c r="D34">
         <v>5</v>
       </c>
       <c r="E34" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>18.48</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
@@ -1135,17 +1129,17 @@
         <v>46247</v>
       </c>
       <c r="B35" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C35">
-        <v>1.25</v>
+        <v>1.41</v>
       </c>
       <c r="D35">
         <v>5</v>
       </c>
       <c r="E35" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>15</v>
+        <v>16.919999999999998</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
@@ -1153,14 +1147,17 @@
         <v>46247</v>
       </c>
       <c r="B36" t="s">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="C36">
+        <v>1.59</v>
       </c>
       <c r="D36">
         <v>5</v>
       </c>
       <c r="E36" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>0</v>
+        <v>19.080000000000002</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
@@ -1168,17 +1165,14 @@
         <v>46247</v>
       </c>
       <c r="B37" t="s">
-        <v>13</v>
-      </c>
-      <c r="C37">
-        <v>1.41</v>
+        <v>14</v>
       </c>
       <c r="D37">
         <v>5</v>
       </c>
       <c r="E37" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>16.919999999999998</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
@@ -1186,17 +1180,17 @@
         <v>46247</v>
       </c>
       <c r="B38" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C38">
-        <v>1.59</v>
+        <v>1.35</v>
       </c>
       <c r="D38">
         <v>5</v>
       </c>
       <c r="E38" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>19.080000000000002</v>
+        <v>16.200000000000003</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
@@ -1204,14 +1198,17 @@
         <v>46247</v>
       </c>
       <c r="B39" t="s">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="C39">
+        <v>1.34</v>
       </c>
       <c r="D39">
         <v>5</v>
       </c>
       <c r="E39" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>0</v>
+        <v>16.080000000000002</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
@@ -1219,17 +1216,17 @@
         <v>46247</v>
       </c>
       <c r="B40" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C40">
-        <v>1.35</v>
+        <v>1.48</v>
       </c>
       <c r="D40">
         <v>5</v>
       </c>
       <c r="E40" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>16.200000000000003</v>
+        <v>17.759999999999998</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
@@ -1237,17 +1234,17 @@
         <v>46247</v>
       </c>
       <c r="B41" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C41">
-        <v>1.34</v>
+        <v>1.3</v>
       </c>
       <c r="D41">
         <v>5</v>
       </c>
       <c r="E41" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>16.080000000000002</v>
+        <v>15.600000000000001</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
@@ -1255,17 +1252,17 @@
         <v>46247</v>
       </c>
       <c r="B42" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C42">
-        <v>1.48</v>
+        <v>1.24</v>
       </c>
       <c r="D42">
         <v>5</v>
       </c>
       <c r="E42" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>17.759999999999998</v>
+        <v>14.879999999999999</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
@@ -1273,17 +1270,14 @@
         <v>46247</v>
       </c>
       <c r="B43" t="s">
-        <v>19</v>
-      </c>
-      <c r="C43">
-        <v>1.3</v>
+        <v>20</v>
       </c>
       <c r="D43">
         <v>5</v>
       </c>
       <c r="E43" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>15.600000000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
@@ -1291,17 +1285,17 @@
         <v>46247</v>
       </c>
       <c r="B44" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C44">
-        <v>1.24</v>
+        <v>1.33</v>
       </c>
       <c r="D44">
         <v>5</v>
       </c>
       <c r="E44" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>14.879999999999999</v>
+        <v>15.96</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
@@ -1309,14 +1303,17 @@
         <v>46247</v>
       </c>
       <c r="B45" t="s">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="C45">
+        <v>1.39</v>
       </c>
       <c r="D45">
         <v>5</v>
       </c>
       <c r="E45" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>0</v>
+        <v>16.68</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
@@ -1324,35 +1321,35 @@
         <v>46247</v>
       </c>
       <c r="B46" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C46">
-        <v>1.33</v>
+        <v>1.42</v>
       </c>
       <c r="D46">
         <v>5</v>
       </c>
       <c r="E46" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>15.96</v>
+        <v>17.04</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" s="2">
         <v>46247</v>
       </c>
-      <c r="B47" t="s">
-        <v>23</v>
+      <c r="B47" s="4" t="s">
+        <v>24</v>
       </c>
       <c r="C47">
-        <v>1.39</v>
+        <v>1.5</v>
       </c>
       <c r="D47">
         <v>5</v>
       </c>
       <c r="E47" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>16.68</v>
+        <v>18</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
@@ -1360,35 +1357,35 @@
         <v>46247</v>
       </c>
       <c r="B48" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C48">
-        <v>1.42</v>
+        <v>1.24</v>
       </c>
       <c r="D48">
         <v>5</v>
       </c>
       <c r="E48" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>17.04</v>
+        <v>14.879999999999999</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" s="2">
         <v>46247</v>
       </c>
-      <c r="B49" s="4" t="s">
-        <v>25</v>
+      <c r="B49" t="s">
+        <v>29</v>
       </c>
       <c r="C49">
-        <v>1.5</v>
+        <v>1.45</v>
       </c>
       <c r="D49">
         <v>5</v>
       </c>
       <c r="E49" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>18</v>
+        <v>17.399999999999999</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
@@ -1399,50 +1396,43 @@
         <v>26</v>
       </c>
       <c r="C50">
-        <v>1.24</v>
+        <v>1.29</v>
       </c>
       <c r="D50">
         <v>5</v>
       </c>
       <c r="E50" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>14.879999999999999</v>
+        <v>15.48</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" s="2">
-        <v>46247</v>
+        <v>46259</v>
       </c>
       <c r="B51" t="s">
-        <v>30</v>
-      </c>
-      <c r="C51">
-        <v>1.45</v>
+        <v>5</v>
       </c>
       <c r="D51">
         <v>5</v>
-      </c>
-      <c r="E51" s="1">
-        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>17.399999999999999</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="2">
-        <v>46247</v>
+        <v>46259</v>
       </c>
       <c r="B52" t="s">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="C52">
-        <v>1.29</v>
+        <v>1.44</v>
       </c>
       <c r="D52">
         <v>5</v>
       </c>
       <c r="E52" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>15.48</v>
+        <v>17.279999999999998</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.3">
@@ -1450,10 +1440,17 @@
         <v>46259</v>
       </c>
       <c r="B53" t="s">
-        <v>5</v>
+        <v>7</v>
+      </c>
+      <c r="C53">
+        <v>1.29</v>
       </c>
       <c r="D53">
         <v>5</v>
+      </c>
+      <c r="E53" s="1">
+        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
+        <v>15.48</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
@@ -1461,17 +1458,17 @@
         <v>46259</v>
       </c>
       <c r="B54" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C54">
-        <v>1.44</v>
+        <v>1.26</v>
       </c>
       <c r="D54">
         <v>5</v>
       </c>
       <c r="E54" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>17.279999999999998</v>
+        <v>15.120000000000001</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.3">
@@ -1479,17 +1476,17 @@
         <v>46259</v>
       </c>
       <c r="B55" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C55">
-        <v>1.29</v>
+        <v>1.38</v>
       </c>
       <c r="D55">
         <v>5</v>
       </c>
       <c r="E55" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>15.48</v>
+        <v>16.559999999999999</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.3">
@@ -1497,17 +1494,17 @@
         <v>46259</v>
       </c>
       <c r="B56" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C56">
-        <v>1.26</v>
+        <v>1.61</v>
       </c>
       <c r="D56">
         <v>5</v>
       </c>
       <c r="E56" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>15.120000000000001</v>
+        <v>19.32</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.3">
@@ -1515,17 +1512,17 @@
         <v>46259</v>
       </c>
       <c r="B57" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C57">
-        <v>1.38</v>
+        <v>1.39</v>
       </c>
       <c r="D57">
         <v>5</v>
       </c>
       <c r="E57" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>16.559999999999999</v>
+        <v>16.68</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.3">
@@ -1533,17 +1530,17 @@
         <v>46259</v>
       </c>
       <c r="B58" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C58">
-        <v>1.61</v>
+        <v>1.17</v>
       </c>
       <c r="D58">
         <v>5</v>
       </c>
       <c r="E58" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>19.32</v>
+        <v>14.04</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.3">
@@ -1551,17 +1548,17 @@
         <v>46259</v>
       </c>
       <c r="B59" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C59">
-        <v>1.31</v>
+        <v>1.56</v>
       </c>
       <c r="D59">
         <v>5</v>
       </c>
       <c r="E59" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>15.72</v>
+        <v>18.72</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.3">
@@ -1569,17 +1566,14 @@
         <v>46259</v>
       </c>
       <c r="B60" t="s">
-        <v>12</v>
-      </c>
-      <c r="C60">
-        <v>1.39</v>
+        <v>14</v>
       </c>
       <c r="D60">
         <v>5</v>
       </c>
       <c r="E60" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>16.68</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.3">
@@ -1587,17 +1581,17 @@
         <v>46259</v>
       </c>
       <c r="B61" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C61">
-        <v>1.17</v>
+        <v>1.35</v>
       </c>
       <c r="D61">
         <v>5</v>
       </c>
       <c r="E61" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>14.04</v>
+        <v>16.200000000000003</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.3">
@@ -1605,17 +1599,17 @@
         <v>46259</v>
       </c>
       <c r="B62" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C62">
-        <v>1.56</v>
+        <v>1.2</v>
       </c>
       <c r="D62">
         <v>5</v>
       </c>
       <c r="E62" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>18.72</v>
+        <v>14.399999999999999</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.3">
@@ -1623,14 +1617,17 @@
         <v>46259</v>
       </c>
       <c r="B63" t="s">
-        <v>15</v>
+        <v>17</v>
+      </c>
+      <c r="C63">
+        <v>1.48</v>
       </c>
       <c r="D63">
         <v>5</v>
       </c>
       <c r="E63" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>0</v>
+        <v>17.759999999999998</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.3">
@@ -1638,17 +1635,17 @@
         <v>46259</v>
       </c>
       <c r="B64" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C64">
-        <v>1.35</v>
+        <v>1.31</v>
       </c>
       <c r="D64">
         <v>5</v>
       </c>
       <c r="E64" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>16.200000000000003</v>
+        <v>15.72</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.3">
@@ -1656,17 +1653,17 @@
         <v>46259</v>
       </c>
       <c r="B65" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C65">
-        <v>1.2</v>
+        <v>1.24</v>
       </c>
       <c r="D65">
         <v>5</v>
       </c>
       <c r="E65" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>14.399999999999999</v>
+        <v>14.879999999999999</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.3">
@@ -1674,17 +1671,17 @@
         <v>46259</v>
       </c>
       <c r="B66" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C66">
-        <v>1.48</v>
+        <v>1.4</v>
       </c>
       <c r="D66">
         <v>5</v>
       </c>
       <c r="E66" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>17.759999999999998</v>
+        <v>16.799999999999997</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.3">
@@ -1692,17 +1689,17 @@
         <v>46259</v>
       </c>
       <c r="B67" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C67">
-        <v>1.31</v>
+        <v>1.42</v>
       </c>
       <c r="D67">
         <v>5</v>
       </c>
       <c r="E67" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>15.72</v>
+        <v>17.04</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.3">
@@ -1710,35 +1707,35 @@
         <v>46259</v>
       </c>
       <c r="B68" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C68">
-        <v>1.24</v>
+        <v>1.28</v>
       </c>
       <c r="D68">
         <v>5</v>
       </c>
       <c r="E68" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>14.879999999999999</v>
+        <v>15.36</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" s="2">
         <v>46259</v>
       </c>
-      <c r="B69" t="s">
-        <v>21</v>
+      <c r="B69" s="4" t="s">
+        <v>24</v>
       </c>
       <c r="C69">
-        <v>1.4</v>
+        <v>1.46</v>
       </c>
       <c r="D69">
         <v>5</v>
       </c>
       <c r="E69" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>16.799999999999997</v>
+        <v>17.52</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.3">
@@ -1746,17 +1743,17 @@
         <v>46259</v>
       </c>
       <c r="B70" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C70">
-        <v>1.42</v>
+        <v>1.33</v>
       </c>
       <c r="D70">
         <v>5</v>
       </c>
       <c r="E70" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>17.04</v>
+        <v>15.96</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.3">
@@ -1764,105 +1761,51 @@
         <v>46259</v>
       </c>
       <c r="B71" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="C71">
-        <v>1.28</v>
+        <v>1.5</v>
       </c>
       <c r="D71">
         <v>5</v>
       </c>
       <c r="E71" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>15.36</v>
+        <v>18</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" s="2">
         <v>46259</v>
       </c>
-      <c r="B72" s="4" t="s">
-        <v>25</v>
+      <c r="B72" t="s">
+        <v>26</v>
       </c>
       <c r="C72">
-        <v>1.46</v>
+        <v>1.4</v>
       </c>
       <c r="D72">
         <v>5</v>
       </c>
       <c r="E72" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>17.52</v>
+        <v>16.799999999999997</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73" s="2">
         <v>46259</v>
       </c>
-      <c r="B73" t="s">
-        <v>26</v>
+      <c r="B73" s="4" t="s">
+        <v>31</v>
       </c>
       <c r="C73">
-        <v>1.33</v>
+        <v>1.41</v>
       </c>
       <c r="D73">
         <v>5</v>
       </c>
       <c r="E73" s="1">
-        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>15.96</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A74" s="2">
-        <v>46259</v>
-      </c>
-      <c r="B74" t="s">
-        <v>30</v>
-      </c>
-      <c r="C74">
-        <v>1.5</v>
-      </c>
-      <c r="D74">
-        <v>5</v>
-      </c>
-      <c r="E74" s="1">
-        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>18</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A75" s="2">
-        <v>46259</v>
-      </c>
-      <c r="B75" t="s">
-        <v>27</v>
-      </c>
-      <c r="C75">
-        <v>1.4</v>
-      </c>
-      <c r="D75">
-        <v>5</v>
-      </c>
-      <c r="E75" s="1">
-        <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
-        <v>16.799999999999997</v>
-      </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A76" s="2">
-        <v>46259</v>
-      </c>
-      <c r="B76" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C76">
-        <v>1.41</v>
-      </c>
-      <c r="D76">
-        <v>5</v>
-      </c>
-      <c r="E76" s="1">
         <f>(Tabla1[[#This Row],[Distancia]]/Tabla1[[#This Row],[Tiempo ]])*60</f>
         <v>16.919999999999998</v>
       </c>

</xml_diff>